<commit_message>
AI Mini Drama: scope TC-389 to the Scene edit page, spec basis check before filing
PDRA questioned DRA262610P0345: PM board 6 「10/12 update - Scene 編輯頁的「地點圖片」」
is the Scene edit page Location thumbnail, not the chat storyboard skeleton, which matches
the Design. TC-389 (both tables) and R-299 now name that screen and record Blocked when it
cannot be reached. An audit of the A2 batch (spec-basis-audit.md) found 4-5 invalid and
11 suspect entries; the skill gains a scope rule in Reading the spec step 4 and a spec
basis check in eBug drafts step 1. Ledger: REQ-054 (A4 full run, was a local REQ-052)
and REQ-055 (this request).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/library/ai-mini-drama/android/cases.xlsx
+++ b/library/ai-mini-drama/android/cases.xlsx
@@ -2042,10 +2042,10 @@
     <t>TC-389</t>
   </si>
   <si>
-    <t>Storyboard generating; a scene with a Location</t>
-  </si>
-  <si>
-    <t>Open that scene's detail while it generates and watch the Location thumbnail</t>
+    <t>Scene detail (Scene edit page) open while that scene's Location image is still generating: the scene regenerated from Edit (TC-070) or updated through Iris (TC-073)</t>
+  </si>
+  <si>
+    <t>Watch the Location thumbnail under the main image until both images finish</t>
   </si>
   <si>
     <t>The Location thumbnail shows a skeleton, then the location image before the main image finishes; the main image keeps its width</t>
@@ -2054,7 +2054,7 @@
     <t>R-299</t>
   </si>
   <si>
-    <t>PM 10/14 board 6; TC-066 notes the Design draws no 「Location」 label</t>
+    <t>PM 10/14 board 6 「10/12 update - Scene 編輯頁的「地點圖片」」: the rule is for the Scene edit page only. The chat storyboard card shows one skeleton loader (Design) and is not this row; if no scene detail can be opened while its Location generates, record Blocked (test-data), not a finding on another screen (Android DRA262610P0345 was filed from that misreading; PDRA 2026-10-29, REQ-055). TC-066 notes the Design draws no 「Location」 label</t>
   </si>
   <si>
     <t>TC-390</t>

</xml_diff>